<commit_message>
Updated BOM and KiCad files
</commit_message>
<xml_diff>
--- a/Docs/V2L Relay Board BOM.xlsx
+++ b/Docs/V2L Relay Board BOM.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="71">
   <si>
     <t>Item #</t>
   </si>
@@ -91,7 +91,7 @@
     <t>MCU Input Driver</t>
   </si>
   <si>
-    <t>2N70000</t>
+    <t>2N7000</t>
   </si>
   <si>
     <t>DigiKey</t>
@@ -127,13 +127,10 @@
     <t>Relay</t>
   </si>
   <si>
-    <t>2071556-8</t>
-  </si>
-  <si>
-    <t>Using "G2RL-1A" in schematic bc no downloadable models</t>
-  </si>
-  <si>
-    <t>https://www.mouser.com/ProductDetail/TE-Connectivity/2071556-8?qs=sGAEpiMZZMtGt%252Bn33CgIP5W55844hwAuTHyZDoDb0Xk%3D</t>
+    <t>G5Q-1A-DC12</t>
+  </si>
+  <si>
+    <t>https://www.mouser.com/ProductDetail/Omron-Electronics/G5Q-1A-DC12?qs=nNiD76Ca0%252Bt4ZP93oe2MyA%3D%3D&amp;srsltid=AfmBOopJJbb029pr-3XQZFCwQl1u7wq2rLvA4L54DUFuBSGrco3OBnPq</t>
   </si>
   <si>
     <t>Switch</t>
@@ -176,6 +173,57 @@
   </si>
   <si>
     <t>https://www.amazon.com/initeq-STM32F103C8T6-Minimum-Development-Programmer/dp/B079B95L9Y?th=1</t>
+  </si>
+  <si>
+    <t>Resistor</t>
+  </si>
+  <si>
+    <t>430 ohms</t>
+  </si>
+  <si>
+    <t>ERA-2ARB431X</t>
+  </si>
+  <si>
+    <t>https://www.mouser.com/ProductDetail/Panasonic/ERA-2ARB431X?qs=sGAEpiMZZMtlubZbdhIBIAJzGQ31d3NR3evwH1klWzI%3D</t>
+  </si>
+  <si>
+    <t>1.8k ohms</t>
+  </si>
+  <si>
+    <t>ERA-6AED182V</t>
+  </si>
+  <si>
+    <t>https://www.mouser.com/ProductDetail/Panasonic/ERA-6AED182V?qs=sGAEpiMZZMtlubZbdhIBINE5Vwz7C5t%2FOQPfWpHRNUY%3D</t>
+  </si>
+  <si>
+    <t>Capacitor</t>
+  </si>
+  <si>
+    <t>0.1uF</t>
+  </si>
+  <si>
+    <t>CL05B104KBD6PJC</t>
+  </si>
+  <si>
+    <t>https://www.mouser.com/ProductDetail/Samsung-Electro-Mechanics/CL05B104KBD6PJC?qs=sGAEpiMZZMsh%252B1woXyUXj%2Fmb4TiHnO1rFKeWMvaPPL8%3D</t>
+  </si>
+  <si>
+    <t>1uF</t>
+  </si>
+  <si>
+    <t>AMK063AC6105MP-F</t>
+  </si>
+  <si>
+    <t>https://www.mouser.com/ProductDetail/TAIYO-YUDEN/AMK063AC6105MP-F?qs=sGAEpiMZZMsh%252B1woXyUXj3HATp5z5h9Ls%2FM2CHI7l3I%3D</t>
+  </si>
+  <si>
+    <t>2.2uF</t>
+  </si>
+  <si>
+    <t>ZRB157R6YA225KE11D</t>
+  </si>
+  <si>
+    <t>https://www.mouser.com/ProductDetail/Murata-Electronics/ZRB157R6YA225KE11D?qs=sGAEpiMZZMsh%252B1woXyUXj%2Fze%252BJJ8bUKCMjpJq3Hfpgk%3D</t>
   </si>
 </sst>
 </file>
@@ -185,7 +233,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <sz val="10.0"/>
       <color rgb="FF000000"/>
@@ -207,6 +255,10 @@
       <u/>
       <color rgb="FF000000"/>
     </font>
+    <font>
+      <u/>
+      <color rgb="FF000000"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -222,7 +274,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -239,9 +291,10 @@
     <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
+    <xf borderId="0" fillId="0" fontId="1" numFmtId="164" xfId="0" applyFont="1" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle xfId="0" name="Normal" builtinId="0"/>
@@ -520,16 +573,17 @@
         <v>13</v>
       </c>
       <c r="E2" s="2">
-        <v>2313.0</v>
+        <v>1756.0</v>
       </c>
       <c r="F2" s="2">
-        <v>9.0</v>
+        <v>16.0</v>
       </c>
       <c r="G2" s="3">
         <v>0.4</v>
       </c>
       <c r="H2" s="3">
-        <v>3.6</v>
+        <f t="shared" ref="H2:H16" si="1">F2*G2</f>
+        <v>6.4</v>
       </c>
       <c r="I2" s="2" t="s">
         <v>14</v>
@@ -553,16 +607,17 @@
         <v>18</v>
       </c>
       <c r="E3" s="2">
-        <v>1607.0</v>
+        <v>1756.0</v>
       </c>
       <c r="F3" s="2">
-        <v>9.0</v>
+        <v>16.0</v>
       </c>
       <c r="G3" s="3">
         <v>0.91</v>
       </c>
       <c r="H3" s="3">
-        <v>8.19</v>
+        <f t="shared" si="1"/>
+        <v>14.56</v>
       </c>
       <c r="I3" s="2" t="s">
         <v>14</v>
@@ -589,13 +644,14 @@
         <v>66223.0</v>
       </c>
       <c r="F4" s="2">
-        <v>9.0</v>
+        <v>16.0</v>
       </c>
       <c r="G4" s="3">
         <v>0.17</v>
       </c>
       <c r="H4" s="3">
-        <v>1.53</v>
+        <f t="shared" si="1"/>
+        <v>2.72</v>
       </c>
       <c r="I4" s="2" t="s">
         <v>14</v>
@@ -622,19 +678,20 @@
         <v>45978.0</v>
       </c>
       <c r="F5" s="2">
-        <v>9.0</v>
+        <v>16.0</v>
       </c>
       <c r="G5" s="3">
         <v>0.65</v>
       </c>
       <c r="H5" s="3">
-        <v>5.85</v>
+        <f t="shared" si="1"/>
+        <v>10.4</v>
       </c>
       <c r="I5" s="2" t="s">
         <v>27</v>
       </c>
       <c r="J5" s="4"/>
-      <c r="K5" s="5" t="s">
+      <c r="K5" s="6" t="s">
         <v>28</v>
       </c>
     </row>
@@ -655,19 +712,20 @@
         <v>387509.0</v>
       </c>
       <c r="F6" s="2">
-        <v>9.0</v>
+        <v>16.0</v>
       </c>
       <c r="G6" s="3">
         <v>0.14</v>
       </c>
       <c r="H6" s="3">
-        <v>1.26</v>
+        <f t="shared" si="1"/>
+        <v>2.24</v>
       </c>
       <c r="I6" s="2" t="s">
         <v>27</v>
       </c>
       <c r="J6" s="4"/>
-      <c r="K6" s="5" t="s">
+      <c r="K6" s="6" t="s">
         <v>32</v>
       </c>
     </row>
@@ -685,22 +743,23 @@
         <v>35</v>
       </c>
       <c r="E7" s="2">
-        <v>17669.0</v>
+        <v>16546.0</v>
       </c>
       <c r="F7" s="2">
-        <v>9.0</v>
+        <v>16.0</v>
       </c>
       <c r="G7" s="3">
         <v>0.18</v>
       </c>
       <c r="H7" s="3">
-        <v>1.62</v>
+        <f t="shared" si="1"/>
+        <v>2.88</v>
       </c>
       <c r="I7" s="2" t="s">
         <v>27</v>
       </c>
       <c r="J7" s="4"/>
-      <c r="K7" s="5" t="s">
+      <c r="K7" s="6" t="s">
         <v>36</v>
       </c>
     </row>
@@ -718,25 +777,24 @@
         <v>38</v>
       </c>
       <c r="E8" s="2">
-        <v>2910.0</v>
+        <v>2201.0</v>
       </c>
       <c r="F8" s="2">
-        <v>9.0</v>
+        <v>16.0</v>
       </c>
       <c r="G8" s="3">
-        <v>1.03</v>
+        <v>1.76</v>
       </c>
       <c r="H8" s="3">
-        <v>9.27</v>
+        <f t="shared" si="1"/>
+        <v>28.16</v>
       </c>
       <c r="I8" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="J8" s="2" t="s">
+      <c r="J8" s="2"/>
+      <c r="K8" s="6" t="s">
         <v>39</v>
-      </c>
-      <c r="K8" s="5" t="s">
-        <v>40</v>
       </c>
     </row>
     <row r="9">
@@ -744,13 +802,13 @@
         <v>8.0</v>
       </c>
       <c r="B9" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="C9" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="C9" s="2" t="s">
+      <c r="D9" s="2" t="s">
         <v>42</v>
-      </c>
-      <c r="D9" s="2" t="s">
-        <v>43</v>
       </c>
       <c r="E9" s="2">
         <v>220.0</v>
@@ -762,16 +820,17 @@
         <v>2.93</v>
       </c>
       <c r="H9" s="3">
+        <f t="shared" si="1"/>
         <v>2.93</v>
       </c>
       <c r="I9" s="2" t="s">
         <v>14</v>
       </c>
       <c r="J9" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="K9" s="5" t="s">
         <v>44</v>
-      </c>
-      <c r="K9" s="5" t="s">
-        <v>45</v>
       </c>
     </row>
     <row r="10">
@@ -779,16 +838,16 @@
         <v>9.0</v>
       </c>
       <c r="B10" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="C10" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="C10" s="2" t="s">
+      <c r="D10" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="D10" s="2" t="s">
-        <v>48</v>
-      </c>
       <c r="E10" s="2">
-        <v>6434.0</v>
+        <v>4353.0</v>
       </c>
       <c r="F10" s="2">
         <v>1.0</v>
@@ -797,14 +856,15 @@
         <v>0.53</v>
       </c>
       <c r="H10" s="3">
+        <f t="shared" si="1"/>
         <v>0.53</v>
       </c>
       <c r="I10" s="2" t="s">
         <v>14</v>
       </c>
       <c r="J10" s="4"/>
-      <c r="K10" s="5" t="s">
-        <v>49</v>
+      <c r="K10" s="6" t="s">
+        <v>48</v>
       </c>
     </row>
     <row r="11">
@@ -812,13 +872,13 @@
         <v>10.0</v>
       </c>
       <c r="B11" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="C11" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="C11" s="2" t="s">
+      <c r="D11" s="2" t="s">
         <v>51</v>
-      </c>
-      <c r="D11" s="2" t="s">
-        <v>52</v>
       </c>
       <c r="E11" s="4"/>
       <c r="F11" s="2">
@@ -828,82 +888,186 @@
         <v>37.99</v>
       </c>
       <c r="H11" s="3">
+        <f t="shared" si="1"/>
         <v>37.99</v>
       </c>
       <c r="I11" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="J11" s="4"/>
       <c r="K11" s="5" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="1">
+        <v>11.0</v>
+      </c>
+      <c r="B12" s="2" t="s">
         <v>54</v>
       </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="4"/>
-      <c r="B12" s="4"/>
-      <c r="C12" s="4"/>
-      <c r="D12" s="4"/>
-      <c r="E12" s="4"/>
-      <c r="F12" s="4"/>
-      <c r="G12" s="4"/>
-      <c r="H12" s="6">
-        <v>72.77</v>
-      </c>
-      <c r="I12" s="4"/>
+      <c r="C12" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="E12" s="2">
+        <v>9652.0</v>
+      </c>
+      <c r="F12" s="2">
+        <v>16.0</v>
+      </c>
+      <c r="G12" s="3">
+        <v>0.53</v>
+      </c>
+      <c r="H12" s="3">
+        <f t="shared" si="1"/>
+        <v>8.48</v>
+      </c>
+      <c r="I12" s="2" t="s">
+        <v>14</v>
+      </c>
       <c r="J12" s="4"/>
-      <c r="K12" s="4"/>
+      <c r="K12" s="6" t="s">
+        <v>57</v>
+      </c>
     </row>
     <row r="13">
-      <c r="A13" s="4"/>
-      <c r="B13" s="4"/>
-      <c r="C13" s="4"/>
-      <c r="D13" s="4"/>
-      <c r="E13" s="4"/>
-      <c r="F13" s="4"/>
-      <c r="G13" s="4"/>
-      <c r="H13" s="4"/>
-      <c r="I13" s="4"/>
+      <c r="A13" s="1">
+        <v>12.0</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="E13" s="2">
+        <v>65824.0</v>
+      </c>
+      <c r="F13" s="2">
+        <v>16.0</v>
+      </c>
+      <c r="G13" s="3">
+        <v>0.28</v>
+      </c>
+      <c r="H13" s="3">
+        <f t="shared" si="1"/>
+        <v>4.48</v>
+      </c>
+      <c r="I13" s="2" t="s">
+        <v>14</v>
+      </c>
       <c r="J13" s="4"/>
-      <c r="K13" s="4"/>
+      <c r="K13" s="6" t="s">
+        <v>60</v>
+      </c>
     </row>
     <row r="14">
-      <c r="A14" s="4"/>
-      <c r="B14" s="4"/>
-      <c r="C14" s="4"/>
-      <c r="D14" s="4"/>
-      <c r="E14" s="4"/>
-      <c r="F14" s="4"/>
-      <c r="G14" s="4"/>
-      <c r="H14" s="4"/>
-      <c r="I14" s="4"/>
+      <c r="A14" s="1">
+        <v>13.0</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="E14" s="2">
+        <v>88313.0</v>
+      </c>
+      <c r="F14" s="2">
+        <v>4.0</v>
+      </c>
+      <c r="G14" s="3">
+        <v>0.26</v>
+      </c>
+      <c r="H14" s="3">
+        <f t="shared" si="1"/>
+        <v>1.04</v>
+      </c>
+      <c r="I14" s="2" t="s">
+        <v>14</v>
+      </c>
       <c r="J14" s="4"/>
-      <c r="K14" s="4"/>
+      <c r="K14" s="6" t="s">
+        <v>64</v>
+      </c>
     </row>
     <row r="15">
-      <c r="A15" s="4"/>
-      <c r="B15" s="4"/>
-      <c r="C15" s="4"/>
-      <c r="D15" s="4"/>
-      <c r="E15" s="4"/>
-      <c r="F15" s="4"/>
-      <c r="G15" s="4"/>
-      <c r="H15" s="4"/>
-      <c r="I15" s="4"/>
+      <c r="A15" s="1">
+        <v>14.0</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="E15" s="2">
+        <v>1047442.0</v>
+      </c>
+      <c r="F15" s="2">
+        <v>1.0</v>
+      </c>
+      <c r="G15" s="3">
+        <v>0.13</v>
+      </c>
+      <c r="H15" s="3">
+        <f t="shared" si="1"/>
+        <v>0.13</v>
+      </c>
+      <c r="I15" s="2" t="s">
+        <v>14</v>
+      </c>
       <c r="J15" s="4"/>
-      <c r="K15" s="4"/>
+      <c r="K15" s="5" t="s">
+        <v>67</v>
+      </c>
     </row>
     <row r="16">
-      <c r="A16" s="4"/>
-      <c r="B16" s="4"/>
-      <c r="C16" s="4"/>
-      <c r="D16" s="4"/>
-      <c r="E16" s="4"/>
-      <c r="F16" s="4"/>
-      <c r="G16" s="4"/>
-      <c r="H16" s="4"/>
-      <c r="I16" s="4"/>
+      <c r="A16" s="1">
+        <v>15.0</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="E16" s="2">
+        <v>23623.0</v>
+      </c>
+      <c r="F16" s="2">
+        <v>1.0</v>
+      </c>
+      <c r="G16" s="3">
+        <v>0.32</v>
+      </c>
+      <c r="H16" s="3">
+        <f t="shared" si="1"/>
+        <v>0.32</v>
+      </c>
+      <c r="I16" s="2" t="s">
+        <v>14</v>
+      </c>
       <c r="J16" s="4"/>
-      <c r="K16" s="4"/>
+      <c r="K16" s="5" t="s">
+        <v>70</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="4"/>
@@ -913,7 +1077,10 @@
       <c r="E17" s="4"/>
       <c r="F17" s="4"/>
       <c r="G17" s="4"/>
-      <c r="H17" s="4"/>
+      <c r="H17" s="7">
+        <f>SUM(H2:H16)</f>
+        <v>123.26</v>
+      </c>
       <c r="I17" s="4"/>
       <c r="J17" s="4"/>
       <c r="K17" s="4"/>
@@ -954,7 +1121,12 @@
     <hyperlink r:id="rId8" ref="K9"/>
     <hyperlink r:id="rId9" ref="K10"/>
     <hyperlink r:id="rId10" ref="K11"/>
+    <hyperlink r:id="rId11" ref="K12"/>
+    <hyperlink r:id="rId12" ref="K13"/>
+    <hyperlink r:id="rId13" ref="K14"/>
+    <hyperlink r:id="rId14" ref="K15"/>
+    <hyperlink r:id="rId15" ref="K16"/>
   </hyperlinks>
-  <drawing r:id="rId11"/>
+  <drawing r:id="rId16"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Updated BOM and PCB WIP
</commit_message>
<xml_diff>
--- a/Docs/V2L Relay Board BOM.xlsx
+++ b/Docs/V2L Relay Board BOM.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="77">
   <si>
     <t>Item #</t>
   </si>
@@ -169,10 +169,13 @@
     <t>STM32F103C8T6 Blue Pill</t>
   </si>
   <si>
-    <t>Amazon</t>
-  </si>
-  <si>
-    <t>https://www.amazon.com/initeq-STM32F103C8T6-Minimum-Development-Programmer/dp/B079B95L9Y?th=1</t>
+    <t>Alibaba</t>
+  </si>
+  <si>
+    <t>From Alibaba</t>
+  </si>
+  <si>
+    <t>https://www.alibaba.com/pla/STM32F103C8T6-STM32-Development-Board-Small-System_1601649660708.html?mark=google_shopping&amp;biz=pla&amp;searchText=specialized+ics&amp;product_id=1601649660708&amp;pcy=us_en&amp;src=sem_ggl&amp;field=UG&amp;from=sem_ggl&amp;cmpgn=22635874527&amp;adgrp=177485315221&amp;fditm=&amp;tgt=pla-2412849993011&amp;locintrst=&amp;locphyscl=9013116&amp;mtchtyp=&amp;ntwrk=g&amp;device=c&amp;dvcmdl=&amp;creative=756472634791&amp;plcmnt=&amp;plcmntcat=&amp;aceid=&amp;position=&amp;gad_source=4&amp;gad_campaignid=22635874527&amp;gbraid=0AAAAAD8m77rpzk9DRFrALpR065MkqAsI0&amp;gclid=Cj0KCQjw39zSBhDhARIsANammDs2s8yDsm1stCvAhAzKVw1i4VKgARMU_ofafcZhB_1cp-UuOXKP4j8aAiSuEALw_wcB</t>
   </si>
   <si>
     <t>Resistor</t>
@@ -224,6 +227,21 @@
   </si>
   <si>
     <t>https://www.mouser.com/ProductDetail/Murata-Electronics/ZRB157R6YA225KE11D?qs=sGAEpiMZZMsh%252B1woXyUXj%2Fze%252BJJ8bUKCMjpJq3Hfpgk%3D</t>
+  </si>
+  <si>
+    <t>Screw Terminal</t>
+  </si>
+  <si>
+    <t>Relay Terminals</t>
+  </si>
+  <si>
+    <t>https://www.mouser.com/en/ProductDetail/Phoenix-Contact/1902547?qs=wd%252Bw3mUqFrmbAnEXicRpKg%3D%3D&amp;mgh=1&amp;utm_id=22303307990&amp;utm_source=google&amp;utm_medium=cpc&amp;utm_marketing_tactic=amercorp&amp;gad_source=1&amp;gad_campaignid=22296748227&amp;gbraid=0AAAAADn_wf2KBwZswlRUL0U2nNuPBI0Pc&amp;gclid=Cj0KCQjw39zSBhDhARIsANammDs7Wjq6U-Xra78lHdGjEQEY_opEn8q122oxnXvx_N0kYB-aah_KvXsaAtFZEALw_wcB</t>
+  </si>
+  <si>
+    <t>Input Terminals</t>
+  </si>
+  <si>
+    <t>https://www.mouser.com/en/ProductDetail/Phoenix-Contact/1729128?qs=GFUSqQMLmmnCBVBY3dts9w%3D%3D&amp;utm_id=22330287750&amp;utm_source=google&amp;utm_medium=cpc&amp;utm_marketing_tactic=amercorp&amp;gad_source=1&amp;gad_campaignid=22330289913&amp;gbraid=0AAAAADn_wf0q7vnWbThmpKjIk7IFUaJ6i&amp;gclid=CjwKCAjwmdLSBhANEiwAkREMNxFfUFPfaCeMHd8kbPxJYRsvg97Utt4Hsjs9mhzjnsqn3OER-xDMuRoCFioQAvD_BwE</t>
   </si>
 </sst>
 </file>
@@ -294,7 +312,9 @@
     <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="164" xfId="0" applyFont="1" applyNumberFormat="1"/>
+    <xf borderId="0" fillId="0" fontId="1" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+      <alignment readingOrder="0"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle xfId="0" name="Normal" builtinId="0"/>
@@ -582,7 +602,7 @@
         <v>0.4</v>
       </c>
       <c r="H2" s="3">
-        <f t="shared" ref="H2:H16" si="1">F2*G2</f>
+        <f t="shared" ref="H2:H10" si="1">F2*G2</f>
         <v>6.4</v>
       </c>
       <c r="I2" s="2" t="s">
@@ -885,18 +905,19 @@
         <v>1.0</v>
       </c>
       <c r="G11" s="3">
-        <v>37.99</v>
+        <v>1.26</v>
       </c>
       <c r="H11" s="3">
-        <f t="shared" si="1"/>
-        <v>37.99</v>
+        <v>1.26</v>
       </c>
       <c r="I11" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="J11" s="4"/>
+      <c r="J11" s="2" t="s">
+        <v>53</v>
+      </c>
       <c r="K11" s="5" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="12">
@@ -904,13 +925,13 @@
         <v>11.0</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="E12" s="2">
         <v>9652.0</v>
@@ -922,7 +943,7 @@
         <v>0.53</v>
       </c>
       <c r="H12" s="3">
-        <f t="shared" si="1"/>
+        <f t="shared" ref="H12:H18" si="2">F12*G12</f>
         <v>8.48</v>
       </c>
       <c r="I12" s="2" t="s">
@@ -930,7 +951,7 @@
       </c>
       <c r="J12" s="4"/>
       <c r="K12" s="6" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="13">
@@ -938,13 +959,13 @@
         <v>12.0</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="E13" s="2">
         <v>65824.0</v>
@@ -956,7 +977,7 @@
         <v>0.28</v>
       </c>
       <c r="H13" s="3">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>4.48</v>
       </c>
       <c r="I13" s="2" t="s">
@@ -964,7 +985,7 @@
       </c>
       <c r="J13" s="4"/>
       <c r="K13" s="6" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
     </row>
     <row r="14">
@@ -972,13 +993,13 @@
         <v>13.0</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="E14" s="2">
         <v>88313.0</v>
@@ -990,7 +1011,7 @@
         <v>0.26</v>
       </c>
       <c r="H14" s="3">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>1.04</v>
       </c>
       <c r="I14" s="2" t="s">
@@ -998,7 +1019,7 @@
       </c>
       <c r="J14" s="4"/>
       <c r="K14" s="6" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
     </row>
     <row r="15">
@@ -1006,13 +1027,13 @@
         <v>14.0</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="E15" s="2">
         <v>1047442.0</v>
@@ -1024,7 +1045,7 @@
         <v>0.13</v>
       </c>
       <c r="H15" s="3">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0.13</v>
       </c>
       <c r="I15" s="2" t="s">
@@ -1032,7 +1053,7 @@
       </c>
       <c r="J15" s="4"/>
       <c r="K15" s="5" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
     </row>
     <row r="16">
@@ -1040,13 +1061,13 @@
         <v>15.0</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="E16" s="2">
         <v>23623.0</v>
@@ -1058,7 +1079,7 @@
         <v>0.32</v>
       </c>
       <c r="H16" s="3">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0.32</v>
       </c>
       <c r="I16" s="2" t="s">
@@ -1066,37 +1087,76 @@
       </c>
       <c r="J16" s="4"/>
       <c r="K16" s="5" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="4"/>
-      <c r="B17" s="4"/>
-      <c r="C17" s="4"/>
-      <c r="D17" s="4"/>
-      <c r="E17" s="4"/>
-      <c r="F17" s="4"/>
-      <c r="G17" s="4"/>
-      <c r="H17" s="7">
-        <f>SUM(H2:H16)</f>
-        <v>123.26</v>
-      </c>
-      <c r="I17" s="4"/>
+      <c r="A17" s="1">
+        <v>16.0</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="D17" s="2">
+        <v>1902547.0</v>
+      </c>
+      <c r="E17" s="2">
+        <v>283.0</v>
+      </c>
+      <c r="F17" s="2">
+        <v>16.0</v>
+      </c>
+      <c r="G17" s="3">
+        <v>1.83</v>
+      </c>
+      <c r="H17" s="3">
+        <f t="shared" si="2"/>
+        <v>29.28</v>
+      </c>
+      <c r="I17" s="2" t="s">
+        <v>14</v>
+      </c>
       <c r="J17" s="4"/>
-      <c r="K17" s="4"/>
+      <c r="K17" s="5" t="s">
+        <v>74</v>
+      </c>
     </row>
     <row r="18">
-      <c r="A18" s="4"/>
-      <c r="B18" s="4"/>
-      <c r="C18" s="4"/>
-      <c r="D18" s="4"/>
-      <c r="E18" s="4"/>
-      <c r="F18" s="4"/>
-      <c r="G18" s="4"/>
-      <c r="H18" s="4"/>
-      <c r="I18" s="4"/>
+      <c r="A18" s="1">
+        <v>17.0</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="D18" s="2">
+        <v>1729128.0</v>
+      </c>
+      <c r="E18" s="2">
+        <v>15528.0</v>
+      </c>
+      <c r="F18" s="2">
+        <v>3.0</v>
+      </c>
+      <c r="G18" s="3">
+        <v>0.95</v>
+      </c>
+      <c r="H18" s="3">
+        <f t="shared" si="2"/>
+        <v>2.85</v>
+      </c>
+      <c r="I18" s="2" t="s">
+        <v>14</v>
+      </c>
       <c r="J18" s="4"/>
-      <c r="K18" s="4"/>
+      <c r="K18" s="5" t="s">
+        <v>76</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="4"/>
@@ -1104,9 +1164,12 @@
       <c r="C19" s="4"/>
       <c r="D19" s="4"/>
       <c r="E19" s="4"/>
-      <c r="F19" s="4"/>
+      <c r="F19" s="2"/>
       <c r="G19" s="4"/>
-      <c r="H19" s="4"/>
+      <c r="H19" s="7">
+        <f>SUM(H2:H18)</f>
+        <v>118.66</v>
+      </c>
       <c r="I19" s="4"/>
     </row>
   </sheetData>
@@ -1126,7 +1189,9 @@
     <hyperlink r:id="rId13" ref="K14"/>
     <hyperlink r:id="rId14" ref="K15"/>
     <hyperlink r:id="rId15" ref="K16"/>
+    <hyperlink r:id="rId16" ref="K17"/>
+    <hyperlink r:id="rId17" ref="K18"/>
   </hyperlinks>
-  <drawing r:id="rId16"/>
+  <drawing r:id="rId18"/>
 </worksheet>
 </file>
</xml_diff>